<commit_message>
Update charts for multiple versions
</commit_message>
<xml_diff>
--- a/2024/day15/data.xlsx
+++ b/2024/day15/data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ΙΣΤΟΧΩΡΟΣ ΣΤΑΤΙΣΤΙΚΗΣ\ΙΣΤΟΧΩΡΟΣ(A1106_SME_18) -ΣΤΟΛΟΣ ΟΧΗΜΑΤΩΝ\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\menexesk\AppData\Local\Microsoft\Windows\INetCache\Content.Outlook\PEC6XILA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE4B3A43-7FF5-4F4F-B896-C6475BB99B8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09E06D88-254E-4863-A974-68197F80FC8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -125,10 +125,10 @@
     <t>Phone : (0030) 213 135 3055</t>
   </si>
   <si>
-    <t xml:space="preserve"> Αυτοκίνητα και μοτοσυκλέτες που  κυκλοφορούσαν  στην Ελλάδα κατά το τέλος των ετών 1985 - 2023.     </t>
+    <t xml:space="preserve"> Αυτοκίνητα και μοτοσυκλέτες που  κυκλοφορούσαν  στην Ελλάδα κατά το τέλος των ετών 1985 - 2025.     </t>
   </si>
   <si>
-    <t>Motor vehicles in operation, by category and use : 1985 - 2023.</t>
+    <t>Motor vehicles in operation, by category and use : 1985 - 2025.</t>
   </si>
 </sst>
 </file>
@@ -179,7 +179,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -302,19 +302,19 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top/>
-      <bottom style="medium">
+      <top style="medium">
         <color indexed="64"/>
-      </bottom>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="medium">
+      <top style="medium">
         <color indexed="64"/>
-      </bottom>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -322,8 +322,39 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
       <top/>
-      <bottom style="medium">
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -332,15 +363,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -359,8 +387,6 @@
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -375,22 +401,43 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -818,7 +865,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V44"/>
+  <dimension ref="A1:W44"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.28515625" customWidth="1"/>
@@ -834,216 +881,224 @@
     <col min="13" max="13" width="9.7109375" customWidth="1"/>
     <col min="14" max="14" width="11" customWidth="1"/>
     <col min="15" max="15" width="9.85546875" customWidth="1"/>
-    <col min="16" max="21" width="9.7109375" customWidth="1"/>
-    <col min="22" max="22" width="16.7109375" customWidth="1"/>
+    <col min="16" max="22" width="9.7109375" customWidth="1"/>
+    <col min="23" max="23" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="33"/>
-      <c r="B1" s="31" t="s">
+    <row r="1" spans="1:23" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="25"/>
+      <c r="B1" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
-      <c r="M1" s="32"/>
-      <c r="N1" s="32"/>
-      <c r="O1" s="32"/>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="32"/>
-      <c r="R1" s="32"/>
-      <c r="S1" s="32"/>
-      <c r="T1" s="32"/>
-      <c r="U1" s="35"/>
-      <c r="V1" s="34"/>
-    </row>
-    <row r="2" spans="1:22" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="26"/>
-      <c r="B2" s="31" t="s">
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
+      <c r="M1" s="41"/>
+      <c r="N1" s="41"/>
+      <c r="O1" s="41"/>
+      <c r="P1" s="41"/>
+      <c r="Q1" s="41"/>
+      <c r="R1" s="41"/>
+      <c r="S1" s="41"/>
+      <c r="T1" s="41"/>
+      <c r="U1" s="41"/>
+      <c r="V1" s="42"/>
+      <c r="W1" s="26"/>
+    </row>
+    <row r="2" spans="1:23" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="23"/>
+      <c r="B2" s="43" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="32"/>
-      <c r="O2" s="32"/>
-      <c r="P2" s="32"/>
-      <c r="Q2" s="32"/>
-      <c r="R2" s="32"/>
-      <c r="S2" s="32"/>
-      <c r="T2" s="32"/>
-      <c r="U2" s="35"/>
-      <c r="V2" s="27"/>
-    </row>
-    <row r="3" spans="1:22" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="25" t="s">
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44"/>
+      <c r="P2" s="44"/>
+      <c r="Q2" s="44"/>
+      <c r="R2" s="44"/>
+      <c r="S2" s="44"/>
+      <c r="T2" s="44"/>
+      <c r="U2" s="44"/>
+      <c r="V2" s="45"/>
+      <c r="W2" s="24"/>
+    </row>
+    <row r="3" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="28">
+      <c r="B3" s="29">
         <v>1985</v>
       </c>
-      <c r="C3" s="29">
+      <c r="C3" s="27">
         <v>1986</v>
       </c>
-      <c r="D3" s="29">
+      <c r="D3" s="27">
         <v>1987</v>
       </c>
-      <c r="E3" s="29">
+      <c r="E3" s="27">
         <v>1988</v>
       </c>
-      <c r="F3" s="29">
+      <c r="F3" s="27">
         <v>1989</v>
       </c>
-      <c r="G3" s="29">
+      <c r="G3" s="27">
         <v>1990</v>
       </c>
-      <c r="H3" s="29">
+      <c r="H3" s="27">
         <v>1991</v>
       </c>
-      <c r="I3" s="29">
+      <c r="I3" s="27">
         <v>1992</v>
       </c>
-      <c r="J3" s="29">
+      <c r="J3" s="27">
         <v>1993</v>
       </c>
-      <c r="K3" s="29">
+      <c r="K3" s="27">
         <v>1994</v>
       </c>
-      <c r="L3" s="29">
+      <c r="L3" s="27">
         <v>1995</v>
       </c>
-      <c r="M3" s="29">
+      <c r="M3" s="27">
         <v>1996</v>
       </c>
-      <c r="N3" s="29">
+      <c r="N3" s="27">
         <v>1997</v>
       </c>
-      <c r="O3" s="29">
+      <c r="O3" s="27">
         <v>1998</v>
       </c>
-      <c r="P3" s="29">
+      <c r="P3" s="27">
         <v>1999</v>
       </c>
-      <c r="Q3" s="29">
+      <c r="Q3" s="27">
         <v>2000</v>
       </c>
-      <c r="R3" s="29">
+      <c r="R3" s="27">
         <v>2001</v>
       </c>
-      <c r="S3" s="29">
+      <c r="S3" s="27">
         <v>2002</v>
       </c>
-      <c r="T3" s="29">
+      <c r="T3" s="27">
         <v>2003</v>
       </c>
-      <c r="U3" s="30">
+      <c r="U3" s="27">
         <v>2004</v>
       </c>
-      <c r="V3" s="21" t="s">
+      <c r="V3" s="28">
+        <v>2005</v>
+      </c>
+      <c r="W3" s="18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="18">
+      <c r="B4" s="30">
         <f t="shared" ref="B4:N4" si="0">SUM(B5,B15)</f>
         <v>2036625</v>
       </c>
-      <c r="C4" s="18">
+      <c r="C4" s="31">
         <f t="shared" si="0"/>
         <v>2170355</v>
       </c>
-      <c r="D4" s="18">
+      <c r="D4" s="31">
         <f t="shared" si="0"/>
         <v>2282494</v>
       </c>
-      <c r="E4" s="18">
+      <c r="E4" s="31">
         <f t="shared" si="0"/>
         <v>2405690</v>
       </c>
-      <c r="F4" s="18">
+      <c r="F4" s="31">
         <f t="shared" si="0"/>
         <v>2569584</v>
       </c>
-      <c r="G4" s="18">
+      <c r="G4" s="31">
         <f t="shared" si="0"/>
         <v>2779976</v>
       </c>
-      <c r="H4" s="18">
+      <c r="H4" s="31">
         <f t="shared" si="0"/>
         <v>2888009</v>
       </c>
-      <c r="I4" s="18">
+      <c r="I4" s="31">
         <f t="shared" si="0"/>
         <v>2989336</v>
       </c>
-      <c r="J4" s="18">
+      <c r="J4" s="31">
         <f t="shared" si="0"/>
         <v>3195324</v>
       </c>
-      <c r="K4" s="18">
+      <c r="K4" s="31">
         <f t="shared" si="0"/>
         <v>3375607</v>
       </c>
-      <c r="L4" s="18">
+      <c r="L4" s="31">
         <f t="shared" si="0"/>
         <v>3588852</v>
       </c>
-      <c r="M4" s="18">
+      <c r="M4" s="31">
         <f t="shared" si="0"/>
         <v>3797234</v>
       </c>
-      <c r="N4" s="18">
+      <c r="N4" s="31">
         <f t="shared" si="0"/>
         <v>4048471</v>
       </c>
-      <c r="O4" s="18">
+      <c r="O4" s="31">
         <v>4323118</v>
       </c>
-      <c r="P4" s="18">
+      <c r="P4" s="31">
         <v>4690412</v>
       </c>
-      <c r="Q4" s="18">
+      <c r="Q4" s="31">
         <v>5060885</v>
       </c>
-      <c r="R4" s="18">
+      <c r="R4" s="31">
         <v>5389996</v>
       </c>
-      <c r="S4" s="3">
+      <c r="S4" s="31">
         <v>5693008</v>
       </c>
-      <c r="T4" s="18">
+      <c r="T4" s="31">
         <v>5967610</v>
       </c>
-      <c r="U4" s="18">
+      <c r="U4" s="31">
         <v>6302033</v>
       </c>
-      <c r="V4" s="15" t="s">
+      <c r="V4" s="32">
+        <v>6640613</v>
+      </c>
+      <c r="W4" s="14" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="s">
+    <row r="5" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="33">
         <f t="shared" ref="B5:N5" si="1">SUM(B6,B9,B12)</f>
         <v>1874330</v>
       </c>
@@ -1116,15 +1171,18 @@
       <c r="U5" s="3">
         <v>5259428</v>
       </c>
-      <c r="V5" s="15" t="s">
+      <c r="V5" s="34">
+        <v>5516441</v>
+      </c>
+      <c r="W5" s="14" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="11" t="s">
+    <row r="6" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="33">
         <f t="shared" ref="B6:N6" si="2">SUM(B7:B8)</f>
         <v>1259335</v>
       </c>
@@ -1197,15 +1255,18 @@
       <c r="U6" s="3">
         <v>4073511</v>
       </c>
-      <c r="V6" s="15" t="s">
+      <c r="V6" s="34">
+        <v>4303129</v>
+      </c>
+      <c r="W6" s="14" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="12" t="s">
+    <row r="7" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="35">
         <v>33265</v>
       </c>
       <c r="C7" s="4">
@@ -1265,15 +1326,18 @@
       <c r="U7" s="4">
         <v>33560</v>
       </c>
-      <c r="V7" s="13" t="s">
+      <c r="V7" s="36">
+        <v>33560</v>
+      </c>
+      <c r="W7" s="12" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="12" t="s">
+    <row r="8" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="35">
         <v>1226070</v>
       </c>
       <c r="C8" s="4">
@@ -1333,15 +1397,18 @@
       <c r="U8" s="4">
         <v>4039951</v>
       </c>
-      <c r="V8" s="13" t="s">
+      <c r="V8" s="36">
+        <v>4269569</v>
+      </c>
+      <c r="W8" s="12" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="11" t="s">
+    <row r="9" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="33">
         <f t="shared" ref="B9:N9" si="3">SUM(B10:B11)</f>
         <v>19234</v>
       </c>
@@ -1414,15 +1481,18 @@
       <c r="U9" s="3">
         <v>26780</v>
       </c>
-      <c r="V9" s="15" t="s">
+      <c r="V9" s="34">
+        <v>26829</v>
+      </c>
+      <c r="W9" s="14" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="13" t="s">
+    <row r="10" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="35">
         <v>13274</v>
       </c>
       <c r="C10" s="4">
@@ -1482,15 +1552,18 @@
       <c r="U10" s="4">
         <v>15069</v>
       </c>
-      <c r="V10" s="13" t="s">
+      <c r="V10" s="36">
+        <v>15069</v>
+      </c>
+      <c r="W10" s="12" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="13" t="s">
+    <row r="11" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B11" s="35">
         <v>5960</v>
       </c>
       <c r="C11" s="4">
@@ -1550,15 +1623,18 @@
       <c r="U11" s="4">
         <v>11711</v>
       </c>
-      <c r="V11" s="13" t="s">
+      <c r="V11" s="36">
+        <v>11760</v>
+      </c>
+      <c r="W11" s="12" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="11" t="s">
+    <row r="12" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" s="33">
         <f t="shared" ref="B12:N12" si="4">SUM(B13:B14)</f>
         <v>595761</v>
       </c>
@@ -1566,7 +1642,7 @@
         <f t="shared" si="4"/>
         <v>622037</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="37">
         <f t="shared" si="4"/>
         <v>650950</v>
       </c>
@@ -1631,15 +1707,18 @@
       <c r="U12" s="3">
         <v>1159137</v>
       </c>
-      <c r="V12" s="15" t="s">
+      <c r="V12" s="34">
+        <v>1186483</v>
+      </c>
+      <c r="W12" s="14" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="13" t="s">
+    <row r="13" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B13" s="35">
         <v>36260</v>
       </c>
       <c r="C13" s="4">
@@ -1699,15 +1778,18 @@
       <c r="U13" s="4">
         <v>36495</v>
       </c>
-      <c r="V13" s="13" t="s">
+      <c r="V13" s="36">
+        <v>36495</v>
+      </c>
+      <c r="W13" s="12" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="13" t="s">
+    <row r="14" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="4">
+      <c r="B14" s="35">
         <v>559501</v>
       </c>
       <c r="C14" s="4">
@@ -1767,15 +1849,18 @@
       <c r="U14" s="4">
         <v>1122642</v>
       </c>
-      <c r="V14" s="13" t="s">
+      <c r="V14" s="36">
+        <v>1149988</v>
+      </c>
+      <c r="W14" s="12" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="11" t="s">
+    <row r="15" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B15" s="33">
         <f t="shared" ref="B15:N15" si="5">SUM(B16:B17)</f>
         <v>162295</v>
       </c>
@@ -1848,15 +1933,18 @@
       <c r="U15" s="3">
         <v>1042605</v>
       </c>
-      <c r="V15" s="15" t="s">
+      <c r="V15" s="34">
+        <v>1124172</v>
+      </c>
+      <c r="W15" s="14" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="13" t="s">
+    <row r="16" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B16" s="35">
         <v>151648</v>
       </c>
       <c r="C16" s="4">
@@ -1916,15 +2004,18 @@
       <c r="U16" s="4">
         <v>1032511</v>
       </c>
-      <c r="V16" s="13" t="s">
+      <c r="V16" s="36">
+        <v>1114099</v>
+      </c>
+      <c r="W16" s="12" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="13" t="s">
+    <row r="17" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B17" s="35">
         <f t="shared" ref="B17:M17" si="6">SUM(B18:B19)</f>
         <v>10647</v>
       </c>
@@ -1997,15 +2088,18 @@
       <c r="U17" s="4">
         <v>10094</v>
       </c>
-      <c r="V17" s="13" t="s">
+      <c r="V17" s="36">
+        <v>10073</v>
+      </c>
+      <c r="W17" s="12" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="13" t="s">
+    <row r="18" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B18" s="35">
         <v>5869</v>
       </c>
       <c r="C18" s="4">
@@ -2065,348 +2159,366 @@
       <c r="U18" s="4">
         <v>5660</v>
       </c>
-      <c r="V18" s="13" t="s">
+      <c r="V18" s="36">
+        <v>5660</v>
+      </c>
+      <c r="W18" s="12" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="13" t="s">
+    <row r="19" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="7">
+      <c r="B19" s="38">
         <v>4778</v>
       </c>
-      <c r="C19" s="7">
+      <c r="C19" s="6">
         <v>4788</v>
       </c>
-      <c r="D19" s="7">
+      <c r="D19" s="6">
         <v>4792</v>
       </c>
-      <c r="E19" s="7">
+      <c r="E19" s="6">
         <v>4795</v>
       </c>
-      <c r="F19" s="7">
+      <c r="F19" s="6">
         <v>4802</v>
       </c>
-      <c r="G19" s="7">
+      <c r="G19" s="6">
         <v>4804</v>
       </c>
-      <c r="H19" s="7">
+      <c r="H19" s="6">
         <v>4811</v>
       </c>
-      <c r="I19" s="7">
+      <c r="I19" s="6">
         <v>4814</v>
       </c>
-      <c r="J19" s="7">
+      <c r="J19" s="6">
         <v>4816</v>
       </c>
-      <c r="K19" s="7">
+      <c r="K19" s="6">
         <v>4815</v>
       </c>
-      <c r="L19" s="7">
+      <c r="L19" s="6">
         <v>4844</v>
       </c>
-      <c r="M19" s="7">
+      <c r="M19" s="6">
         <v>4814</v>
       </c>
-      <c r="N19" s="7">
+      <c r="N19" s="6">
         <v>4784</v>
       </c>
-      <c r="O19" s="7">
+      <c r="O19" s="6">
         <v>4768</v>
       </c>
-      <c r="P19" s="7">
+      <c r="P19" s="6">
         <v>4757</v>
       </c>
-      <c r="Q19" s="7">
+      <c r="Q19" s="6">
         <v>4730</v>
       </c>
-      <c r="R19" s="7">
+      <c r="R19" s="6">
         <v>4661</v>
       </c>
-      <c r="S19" s="7">
+      <c r="S19" s="6">
         <v>4557</v>
       </c>
-      <c r="T19" s="7">
+      <c r="T19" s="6">
         <v>4498</v>
       </c>
-      <c r="U19" s="19">
+      <c r="U19" s="6">
         <v>4434</v>
       </c>
-      <c r="V19" s="13" t="s">
+      <c r="V19" s="39">
+        <v>4413</v>
+      </c>
+      <c r="W19" s="12" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:22" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="16"/>
-      <c r="V20" s="16"/>
-    </row>
-    <row r="21" spans="1:22" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="20" t="s">
+    <row r="20" spans="1:23" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="15"/>
+      <c r="W20" s="15"/>
+    </row>
+    <row r="21" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="22">
-        <v>2005</v>
-      </c>
-      <c r="C21" s="23">
+      <c r="B21" s="19">
         <v>2006</v>
       </c>
-      <c r="D21" s="23">
+      <c r="C21" s="20">
         <v>2007</v>
       </c>
-      <c r="E21" s="23">
+      <c r="D21" s="20">
         <v>2008</v>
       </c>
-      <c r="F21" s="23">
+      <c r="E21" s="20">
         <v>2009</v>
       </c>
-      <c r="G21" s="23">
+      <c r="F21" s="20">
         <v>2010</v>
       </c>
-      <c r="H21" s="23">
+      <c r="G21" s="20">
         <v>2011</v>
       </c>
-      <c r="I21" s="23">
+      <c r="H21" s="20">
         <v>2012</v>
       </c>
-      <c r="J21" s="23">
+      <c r="I21" s="20">
         <v>2013</v>
       </c>
-      <c r="K21" s="23">
+      <c r="J21" s="20">
         <v>2014</v>
       </c>
-      <c r="L21" s="23">
+      <c r="K21" s="20">
         <v>2015</v>
       </c>
-      <c r="M21" s="23">
+      <c r="L21" s="20">
         <v>2016</v>
       </c>
-      <c r="N21" s="23">
+      <c r="M21" s="20">
         <v>2017</v>
       </c>
-      <c r="O21" s="23">
+      <c r="N21" s="20">
         <v>2018</v>
       </c>
-      <c r="P21" s="23">
+      <c r="O21" s="20">
         <v>2019</v>
       </c>
-      <c r="Q21" s="23">
+      <c r="P21" s="20">
         <v>2020</v>
       </c>
-      <c r="R21" s="23">
+      <c r="Q21" s="20">
         <v>2021</v>
       </c>
-      <c r="S21" s="23">
+      <c r="R21" s="20">
         <v>2022</v>
       </c>
-      <c r="T21" s="23">
+      <c r="S21" s="20">
         <v>2023</v>
       </c>
-      <c r="U21" s="24"/>
-      <c r="V21" s="21" t="s">
+      <c r="T21" s="20">
+        <v>2024</v>
+      </c>
+      <c r="U21" s="20">
+        <v>2025</v>
+      </c>
+      <c r="V21" s="21"/>
+      <c r="W21" s="18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="10" t="s">
+    <row r="22" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B22" s="18">
-        <v>6640613</v>
+      <c r="B22" s="3">
+        <v>6995659</v>
       </c>
       <c r="C22" s="3">
-        <v>6995659</v>
+        <v>7380265</v>
       </c>
       <c r="D22" s="3">
-        <v>7380265</v>
+        <v>7729262</v>
       </c>
       <c r="E22" s="3">
-        <v>7729262</v>
+        <v>7910565</v>
       </c>
       <c r="F22" s="3">
-        <v>7910565</v>
+        <v>8062085</v>
       </c>
       <c r="G22" s="3">
-        <v>8062085</v>
+        <v>8086910</v>
       </c>
       <c r="H22" s="3">
-        <v>8086910</v>
+        <v>8069872</v>
       </c>
       <c r="I22" s="3">
-        <v>8069872</v>
+        <v>8035423</v>
       </c>
       <c r="J22" s="3">
-        <v>8035423</v>
+        <v>8048438</v>
       </c>
       <c r="K22" s="3">
-        <v>8048438</v>
+        <v>8076431</v>
       </c>
       <c r="L22" s="3">
-        <v>8076431</v>
+        <v>8172948</v>
       </c>
       <c r="M22" s="3">
-        <v>8172948</v>
+        <v>8262896</v>
       </c>
       <c r="N22" s="3">
-        <v>8262896</v>
+        <v>8236637</v>
       </c>
       <c r="O22" s="3">
-        <v>8236637</v>
+        <v>8402294</v>
       </c>
       <c r="P22" s="3">
-        <v>8402294</v>
+        <v>8530050</v>
       </c>
       <c r="Q22" s="3">
-        <v>8530050</v>
+        <v>8698421</v>
       </c>
       <c r="R22" s="3">
-        <v>8698421</v>
+        <v>8882981</v>
       </c>
       <c r="S22" s="3">
-        <v>8882981</v>
+        <v>9107496</v>
       </c>
       <c r="T22" s="3">
-        <v>9107496</v>
-      </c>
-      <c r="U22" s="3"/>
-      <c r="V22" s="15" t="s">
+        <v>9343429</v>
+      </c>
+      <c r="U22" s="3">
+        <v>9592149</v>
+      </c>
+      <c r="V22" s="3"/>
+      <c r="W22" s="14" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="11" t="s">
+    <row r="23" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="10" t="s">
         <v>14</v>
       </c>
       <c r="B23" s="3">
-        <v>5516441</v>
+        <v>5789843</v>
       </c>
       <c r="C23" s="3">
-        <v>5789843</v>
+        <v>6081577</v>
       </c>
       <c r="D23" s="3">
-        <v>6081577</v>
+        <v>6340655</v>
       </c>
       <c r="E23" s="3">
-        <v>6340655</v>
+        <v>6461714</v>
       </c>
       <c r="F23" s="3">
-        <v>6461714</v>
+        <v>6562952</v>
       </c>
       <c r="G23" s="3">
-        <v>6562952</v>
+        <v>6552008</v>
       </c>
       <c r="H23" s="3">
-        <v>6552008</v>
+        <v>6513437</v>
       </c>
       <c r="I23" s="3">
-        <v>6513437</v>
+        <v>6466827</v>
       </c>
       <c r="J23" s="3">
-        <v>6466827</v>
+        <v>6455509</v>
       </c>
       <c r="K23" s="3">
-        <v>6455509</v>
+        <v>6456810</v>
       </c>
       <c r="L23" s="3">
-        <v>6456810</v>
+        <v>6519420</v>
       </c>
       <c r="M23" s="3">
-        <v>6519420</v>
+        <v>6606239</v>
       </c>
       <c r="N23" s="3">
-        <v>6606239</v>
+        <v>6653146</v>
       </c>
       <c r="O23" s="3">
-        <v>6653146</v>
+        <v>6792371</v>
       </c>
       <c r="P23" s="3">
-        <v>6792371</v>
+        <v>6892442</v>
       </c>
       <c r="Q23" s="3">
-        <v>6892442</v>
+        <v>7022617</v>
       </c>
       <c r="R23" s="3">
-        <v>7022617</v>
+        <v>7158543</v>
       </c>
       <c r="S23" s="3">
-        <v>7158543</v>
+        <v>7325474</v>
       </c>
       <c r="T23" s="3">
-        <v>7325474</v>
-      </c>
-      <c r="U23" s="3"/>
-      <c r="V23" s="15" t="s">
+        <v>7491809</v>
+      </c>
+      <c r="U23" s="3">
+        <v>7670256</v>
+      </c>
+      <c r="V23" s="3"/>
+      <c r="W23" s="14" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="11" t="s">
+    <row r="24" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="10" t="s">
         <v>15</v>
       </c>
       <c r="B24" s="3">
-        <v>4303129</v>
+        <v>4543016</v>
       </c>
       <c r="C24" s="3">
-        <v>4543016</v>
+        <v>4798530</v>
       </c>
       <c r="D24" s="3">
-        <v>4798530</v>
+        <v>5023944</v>
       </c>
       <c r="E24" s="3">
-        <v>5023944</v>
+        <v>5131960</v>
       </c>
       <c r="F24" s="3">
-        <v>5131960</v>
+        <v>5216873</v>
       </c>
       <c r="G24" s="3">
-        <v>5216873</v>
+        <v>5203591</v>
       </c>
       <c r="H24" s="3">
-        <v>5203591</v>
+        <v>5167557</v>
       </c>
       <c r="I24" s="3">
-        <v>5167557</v>
+        <v>5124208</v>
       </c>
       <c r="J24" s="3">
-        <v>5124208</v>
+        <v>5110873</v>
       </c>
       <c r="K24" s="3">
-        <v>5110873</v>
+        <v>5107620</v>
       </c>
       <c r="L24" s="3">
-        <v>5107620</v>
+        <v>5160056</v>
       </c>
       <c r="M24" s="3">
-        <v>5160056</v>
+        <v>5235928</v>
       </c>
       <c r="N24" s="3">
-        <v>5235928</v>
+        <v>5282695</v>
       </c>
       <c r="O24" s="3">
-        <v>5282695</v>
+        <v>5406551</v>
       </c>
       <c r="P24" s="3">
-        <v>5406551</v>
+        <v>5492176</v>
       </c>
       <c r="Q24" s="3">
-        <v>5492176</v>
+        <v>5604192</v>
       </c>
       <c r="R24" s="3">
-        <v>5604192</v>
+        <v>5726012</v>
       </c>
       <c r="S24" s="3">
-        <v>5726012</v>
+        <v>5877759</v>
       </c>
       <c r="T24" s="3">
-        <v>5877759</v>
-      </c>
-      <c r="U24" s="3"/>
-      <c r="V24" s="15" t="s">
+        <v>6027946</v>
+      </c>
+      <c r="U24" s="3">
+        <v>6188525</v>
+      </c>
+      <c r="V24" s="3"/>
+      <c r="W24" s="14" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="12" t="s">
+    <row r="25" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="11" t="s">
         <v>16</v>
       </c>
       <c r="B25" s="4">
@@ -2466,145 +2578,154 @@
       <c r="T25" s="4">
         <v>33560</v>
       </c>
-      <c r="U25" s="4"/>
-      <c r="V25" s="13" t="s">
+      <c r="U25" s="4">
+        <v>33560</v>
+      </c>
+      <c r="V25" s="4"/>
+      <c r="W25" s="12" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="12" t="s">
+    <row r="26" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="11" t="s">
         <v>17</v>
       </c>
       <c r="B26" s="4">
-        <v>4269569</v>
+        <v>4509456</v>
       </c>
       <c r="C26" s="4">
-        <v>4509456</v>
+        <v>4764970</v>
       </c>
       <c r="D26" s="4">
-        <v>4764970</v>
+        <v>4990384</v>
       </c>
       <c r="E26" s="4">
-        <v>4990384</v>
+        <v>5098400</v>
       </c>
       <c r="F26" s="4">
-        <v>5098400</v>
+        <v>5183313</v>
       </c>
       <c r="G26" s="4">
-        <v>5183313</v>
+        <v>5170031</v>
       </c>
       <c r="H26" s="4">
-        <v>5170031</v>
+        <v>5133997</v>
       </c>
       <c r="I26" s="4">
-        <v>5133997</v>
+        <v>5090648</v>
       </c>
       <c r="J26" s="4">
-        <v>5090648</v>
+        <v>5077313</v>
       </c>
       <c r="K26" s="4">
-        <v>5077313</v>
+        <v>5074060</v>
       </c>
       <c r="L26" s="4">
-        <v>5074060</v>
+        <v>5126496</v>
       </c>
       <c r="M26" s="4">
-        <v>5126496</v>
+        <v>5202368</v>
       </c>
       <c r="N26" s="4">
-        <v>5202368</v>
+        <v>5249135</v>
       </c>
       <c r="O26" s="4">
-        <v>5249135</v>
+        <v>5372991</v>
       </c>
       <c r="P26" s="4">
-        <v>5372991</v>
+        <v>5458616</v>
       </c>
       <c r="Q26" s="4">
-        <v>5458616</v>
+        <v>5570632</v>
       </c>
       <c r="R26" s="4">
-        <v>5570632</v>
+        <v>5692452</v>
       </c>
       <c r="S26" s="4">
-        <v>5692452</v>
+        <v>5844199</v>
       </c>
       <c r="T26" s="4">
-        <v>5844199</v>
-      </c>
-      <c r="U26" s="4"/>
-      <c r="V26" s="13" t="s">
+        <v>5994386</v>
+      </c>
+      <c r="U26" s="4">
+        <v>6154965</v>
+      </c>
+      <c r="V26" s="4"/>
+      <c r="W26" s="12" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="11" t="s">
+    <row r="27" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="10" t="s">
         <v>18</v>
       </c>
       <c r="B27" s="3">
-        <v>26829</v>
+        <v>26938</v>
       </c>
       <c r="C27" s="3">
-        <v>26938</v>
+        <v>27102</v>
       </c>
       <c r="D27" s="3">
-        <v>27102</v>
+        <v>27186</v>
       </c>
       <c r="E27" s="3">
-        <v>27186</v>
+        <v>27324</v>
       </c>
       <c r="F27" s="3">
-        <v>27324</v>
+        <v>27311</v>
       </c>
       <c r="G27" s="3">
-        <v>27311</v>
+        <v>27121</v>
       </c>
       <c r="H27" s="3">
-        <v>27121</v>
+        <v>26962</v>
       </c>
       <c r="I27" s="3">
-        <v>26962</v>
+        <v>26783</v>
       </c>
       <c r="J27" s="3">
-        <v>26783</v>
+        <v>26691</v>
       </c>
       <c r="K27" s="3">
-        <v>26691</v>
+        <v>26586</v>
       </c>
       <c r="L27" s="3">
-        <v>26586</v>
+        <v>26541</v>
       </c>
       <c r="M27" s="3">
-        <v>26541</v>
+        <v>26481</v>
       </c>
       <c r="N27" s="3">
-        <v>26481</v>
+        <v>26389</v>
       </c>
       <c r="O27" s="3">
-        <v>26389</v>
+        <v>26479</v>
       </c>
       <c r="P27" s="3">
-        <v>26479</v>
+        <v>26539</v>
       </c>
       <c r="Q27" s="3">
-        <v>26539</v>
+        <v>26584</v>
       </c>
       <c r="R27" s="3">
-        <v>26584</v>
+        <v>26560</v>
       </c>
       <c r="S27" s="3">
-        <v>26560</v>
+        <v>26636</v>
       </c>
       <c r="T27" s="3">
-        <v>26636</v>
-      </c>
-      <c r="U27" s="3"/>
-      <c r="V27" s="15" t="s">
+        <v>26566</v>
+      </c>
+      <c r="U27" s="3">
+        <v>26544</v>
+      </c>
+      <c r="V27" s="3"/>
+      <c r="W27" s="14" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="13" t="s">
+    <row r="28" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="12" t="s">
         <v>19</v>
       </c>
       <c r="B28" s="4">
@@ -2664,145 +2785,154 @@
       <c r="T28" s="4">
         <v>15069</v>
       </c>
-      <c r="U28" s="4"/>
-      <c r="V28" s="13" t="s">
+      <c r="U28" s="4">
+        <v>15069</v>
+      </c>
+      <c r="V28" s="4"/>
+      <c r="W28" s="12" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="13" t="s">
+    <row r="29" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="12" t="s">
         <v>20</v>
       </c>
       <c r="B29" s="4">
-        <v>11760</v>
+        <v>11869</v>
       </c>
       <c r="C29" s="4">
-        <v>11869</v>
+        <v>12033</v>
       </c>
       <c r="D29" s="4">
-        <v>12033</v>
+        <v>12117</v>
       </c>
       <c r="E29" s="4">
-        <v>12117</v>
+        <v>12255</v>
       </c>
       <c r="F29" s="4">
-        <v>12255</v>
+        <v>12242</v>
       </c>
       <c r="G29" s="4">
-        <v>12242</v>
+        <v>12052</v>
       </c>
       <c r="H29" s="4">
-        <v>12052</v>
+        <v>11893</v>
       </c>
       <c r="I29" s="4">
-        <v>11893</v>
+        <v>11714</v>
       </c>
       <c r="J29" s="4">
-        <v>11714</v>
+        <v>11622</v>
       </c>
       <c r="K29" s="4">
-        <v>11622</v>
+        <v>11517</v>
       </c>
       <c r="L29" s="4">
-        <v>11517</v>
+        <v>11472</v>
       </c>
       <c r="M29" s="4">
-        <v>11472</v>
+        <v>11412</v>
       </c>
       <c r="N29" s="4">
-        <v>11412</v>
+        <v>11320</v>
       </c>
       <c r="O29" s="4">
-        <v>11320</v>
+        <v>11410</v>
       </c>
       <c r="P29" s="4">
-        <v>11410</v>
+        <v>11470</v>
       </c>
       <c r="Q29" s="4">
-        <v>11470</v>
+        <v>11515</v>
       </c>
       <c r="R29" s="4">
-        <v>11515</v>
+        <v>11491</v>
       </c>
       <c r="S29" s="4">
-        <v>11491</v>
+        <v>11567</v>
       </c>
       <c r="T29" s="4">
-        <v>11567</v>
-      </c>
-      <c r="U29" s="4"/>
-      <c r="V29" s="13" t="s">
+        <v>11497</v>
+      </c>
+      <c r="U29" s="4">
+        <v>11475</v>
+      </c>
+      <c r="V29" s="4"/>
+      <c r="W29" s="12" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="11" t="s">
+    <row r="30" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B30" s="3">
-        <v>1186483</v>
+        <v>1219889</v>
       </c>
       <c r="C30" s="3">
-        <v>1219889</v>
+        <v>1255945</v>
       </c>
       <c r="D30" s="3">
-        <v>1255945</v>
+        <v>1289525</v>
       </c>
       <c r="E30" s="3">
-        <v>1289525</v>
+        <v>1302430</v>
       </c>
       <c r="F30" s="3">
-        <v>1302430</v>
+        <v>1318768</v>
       </c>
       <c r="G30" s="3">
-        <v>1318768</v>
+        <v>1321296</v>
       </c>
       <c r="H30" s="3">
-        <v>1321296</v>
+        <v>1318918</v>
       </c>
       <c r="I30" s="3">
-        <v>1318918</v>
+        <v>1315836</v>
       </c>
       <c r="J30" s="3">
-        <v>1315836</v>
+        <v>1317945</v>
       </c>
       <c r="K30" s="3">
-        <v>1317945</v>
+        <v>1322604</v>
       </c>
       <c r="L30" s="3">
-        <v>1322604</v>
+        <v>1332823</v>
       </c>
       <c r="M30" s="3">
-        <v>1332823</v>
+        <v>1343830</v>
       </c>
       <c r="N30" s="3">
-        <v>1343830</v>
+        <v>1344062</v>
       </c>
       <c r="O30" s="3">
-        <v>1344062</v>
+        <v>1359341</v>
       </c>
       <c r="P30" s="3">
-        <v>1359341</v>
+        <v>1373727</v>
       </c>
       <c r="Q30" s="3">
-        <v>1373727</v>
+        <v>1391841</v>
       </c>
       <c r="R30" s="3">
-        <v>1391841</v>
+        <v>1405971</v>
       </c>
       <c r="S30" s="3">
-        <v>1405971</v>
+        <v>1421079</v>
       </c>
       <c r="T30" s="3">
-        <v>1421079</v>
-      </c>
-      <c r="U30" s="3"/>
-      <c r="V30" s="15" t="s">
+        <v>1437297</v>
+      </c>
+      <c r="U30" s="3">
+        <v>1455187</v>
+      </c>
+      <c r="V30" s="3"/>
+      <c r="W30" s="14" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="13" t="s">
+    <row r="31" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="12" t="s">
         <v>22</v>
       </c>
       <c r="B31" s="4">
@@ -2862,277 +2992,292 @@
       <c r="T31" s="4">
         <v>36495</v>
       </c>
-      <c r="U31" s="4"/>
-      <c r="V31" s="13" t="s">
+      <c r="U31" s="4">
+        <v>36495</v>
+      </c>
+      <c r="V31" s="4"/>
+      <c r="W31" s="12" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="13" t="s">
+    <row r="32" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="12" t="s">
         <v>20</v>
       </c>
       <c r="B32" s="4">
-        <v>1149988</v>
+        <v>1183394</v>
       </c>
       <c r="C32" s="4">
-        <v>1183394</v>
+        <v>1219450</v>
       </c>
       <c r="D32" s="4">
-        <v>1219450</v>
+        <v>1253030</v>
       </c>
       <c r="E32" s="4">
-        <v>1253030</v>
+        <v>1265935</v>
       </c>
       <c r="F32" s="4">
-        <v>1265935</v>
+        <v>1282273</v>
       </c>
       <c r="G32" s="4">
-        <v>1282273</v>
+        <v>1284801</v>
       </c>
       <c r="H32" s="4">
-        <v>1284801</v>
+        <v>1282423</v>
       </c>
       <c r="I32" s="4">
-        <v>1282423</v>
+        <v>1279341</v>
       </c>
       <c r="J32" s="4">
-        <v>1279341</v>
+        <v>1281450</v>
       </c>
       <c r="K32" s="4">
-        <v>1281450</v>
+        <v>1286109</v>
       </c>
       <c r="L32" s="4">
-        <v>1286109</v>
+        <v>1296328</v>
       </c>
       <c r="M32" s="4">
-        <v>1296328</v>
+        <v>1307335</v>
       </c>
       <c r="N32" s="4">
-        <v>1307335</v>
+        <v>1307567</v>
       </c>
       <c r="O32" s="4">
-        <v>1307567</v>
+        <v>1322846</v>
       </c>
       <c r="P32" s="4">
-        <v>1322846</v>
+        <v>1337232</v>
       </c>
       <c r="Q32" s="4">
-        <v>1337232</v>
+        <v>1355346</v>
       </c>
       <c r="R32" s="4">
-        <v>1355346</v>
+        <v>1369476</v>
       </c>
       <c r="S32" s="4">
-        <v>1369476</v>
+        <v>1384584</v>
       </c>
       <c r="T32" s="4">
-        <v>1384584</v>
-      </c>
-      <c r="U32" s="4"/>
-      <c r="V32" s="13" t="s">
+        <v>1400802</v>
+      </c>
+      <c r="U32" s="4">
+        <v>1418692</v>
+      </c>
+      <c r="V32" s="4"/>
+      <c r="W32" s="12" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="11" t="s">
+    <row r="33" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="10" t="s">
         <v>23</v>
       </c>
       <c r="B33" s="3">
-        <v>1124172</v>
+        <v>1205816</v>
       </c>
       <c r="C33" s="3">
-        <v>1205816</v>
+        <v>1298688</v>
       </c>
       <c r="D33" s="3">
-        <v>1298688</v>
+        <v>1388607</v>
       </c>
       <c r="E33" s="3">
-        <v>1388607</v>
+        <v>1448851</v>
       </c>
       <c r="F33" s="3">
-        <v>1448851</v>
+        <v>1499133</v>
       </c>
       <c r="G33" s="3">
-        <v>1499133</v>
+        <v>1534902</v>
       </c>
       <c r="H33" s="3">
-        <v>1534902</v>
+        <v>1556435</v>
       </c>
       <c r="I33" s="3">
-        <v>1556435</v>
+        <v>1568596</v>
       </c>
       <c r="J33" s="3">
-        <v>1568596</v>
+        <v>1592929</v>
       </c>
       <c r="K33" s="3">
-        <v>1592929</v>
+        <v>1619621</v>
       </c>
       <c r="L33" s="3">
-        <v>1619621</v>
+        <v>1653528</v>
       </c>
       <c r="M33" s="3">
-        <v>1653528</v>
+        <v>1656657</v>
       </c>
       <c r="N33" s="3">
-        <v>1656657</v>
+        <v>1583491</v>
       </c>
       <c r="O33" s="3">
-        <v>1583491</v>
+        <v>1609923</v>
       </c>
       <c r="P33" s="3">
-        <v>1609923</v>
+        <v>1637608</v>
       </c>
       <c r="Q33" s="3">
-        <v>1637608</v>
+        <v>1675804</v>
       </c>
       <c r="R33" s="3">
-        <v>1675804</v>
+        <v>1724438</v>
       </c>
       <c r="S33" s="3">
-        <v>1724438</v>
+        <v>1782022</v>
       </c>
       <c r="T33" s="3">
-        <v>1782022</v>
-      </c>
-      <c r="U33" s="3"/>
-      <c r="V33" s="15" t="s">
+        <v>1851620</v>
+      </c>
+      <c r="U33" s="3">
+        <v>1921893</v>
+      </c>
+      <c r="V33" s="3"/>
+      <c r="W33" s="14" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="13" t="s">
+    <row r="34" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="12" t="s">
         <v>24</v>
       </c>
       <c r="B34" s="4">
-        <v>1114099</v>
+        <v>1195732</v>
       </c>
       <c r="C34" s="4">
-        <v>1195732</v>
+        <v>1288585</v>
       </c>
       <c r="D34" s="4">
-        <v>1288585</v>
+        <v>1378492</v>
       </c>
       <c r="E34" s="4">
-        <v>1378492</v>
+        <v>1438713</v>
       </c>
       <c r="F34" s="4">
-        <v>1438713</v>
+        <v>1488995</v>
       </c>
       <c r="G34" s="4">
-        <v>1488995</v>
+        <v>1524768</v>
       </c>
       <c r="H34" s="4">
-        <v>1524768</v>
+        <v>1546306</v>
       </c>
       <c r="I34" s="4">
-        <v>1546306</v>
+        <v>1558474</v>
       </c>
       <c r="J34" s="4">
-        <v>1558474</v>
+        <v>1582818</v>
       </c>
       <c r="K34" s="4">
-        <v>1582818</v>
+        <v>1609512</v>
       </c>
       <c r="L34" s="4">
-        <v>1609512</v>
+        <v>1643421</v>
       </c>
       <c r="M34" s="4">
-        <v>1643421</v>
+        <v>1646558</v>
       </c>
       <c r="N34" s="4">
-        <v>1646558</v>
+        <v>1573423</v>
       </c>
       <c r="O34" s="4">
-        <v>1573423</v>
+        <v>1599857</v>
       </c>
       <c r="P34" s="4">
-        <v>1599857</v>
+        <v>1627537</v>
       </c>
       <c r="Q34" s="4">
-        <v>1627537</v>
+        <v>1665706</v>
       </c>
       <c r="R34" s="4">
-        <v>1665706</v>
+        <v>1714317</v>
       </c>
       <c r="S34" s="4">
-        <v>1714317</v>
+        <v>1771799</v>
       </c>
       <c r="T34" s="4">
-        <v>1771799</v>
-      </c>
-      <c r="U34" s="4"/>
-      <c r="V34" s="13" t="s">
+        <v>1841304</v>
+      </c>
+      <c r="U34" s="4">
+        <v>1911519</v>
+      </c>
+      <c r="V34" s="4"/>
+      <c r="W34" s="12" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="35" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="13" t="s">
+    <row r="35" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="12" t="s">
         <v>25</v>
       </c>
       <c r="B35" s="4">
-        <v>10073</v>
+        <v>10084</v>
       </c>
       <c r="C35" s="4">
-        <v>10084</v>
+        <v>10103</v>
       </c>
       <c r="D35" s="4">
-        <v>10103</v>
+        <v>10115</v>
       </c>
       <c r="E35" s="4">
-        <v>10115</v>
+        <v>10138</v>
       </c>
       <c r="F35" s="4">
         <v>10138</v>
       </c>
       <c r="G35" s="4">
-        <v>10138</v>
+        <v>10134</v>
       </c>
       <c r="H35" s="4">
-        <v>10134</v>
+        <v>10129</v>
       </c>
       <c r="I35" s="4">
-        <v>10129</v>
+        <v>10122</v>
       </c>
       <c r="J35" s="4">
-        <v>10122</v>
+        <v>10111</v>
       </c>
       <c r="K35" s="4">
-        <v>10111</v>
+        <v>10109</v>
       </c>
       <c r="L35" s="4">
-        <v>10109</v>
+        <v>10107</v>
       </c>
       <c r="M35" s="4">
-        <v>10107</v>
+        <v>10099</v>
       </c>
       <c r="N35" s="4">
-        <v>10099</v>
+        <v>10068</v>
       </c>
       <c r="O35" s="4">
-        <v>10068</v>
+        <v>10066</v>
       </c>
       <c r="P35" s="4">
-        <v>10066</v>
+        <v>10071</v>
       </c>
       <c r="Q35" s="4">
-        <v>10071</v>
+        <v>10098</v>
       </c>
       <c r="R35" s="4">
-        <v>10098</v>
+        <v>10121</v>
       </c>
       <c r="S35" s="4">
-        <v>10121</v>
+        <v>10223</v>
       </c>
       <c r="T35" s="4">
-        <v>10223</v>
-      </c>
-      <c r="U35" s="4"/>
-      <c r="V35" s="13" t="s">
+        <v>10316</v>
+      </c>
+      <c r="U35" s="4">
+        <v>10374</v>
+      </c>
+      <c r="V35" s="4"/>
+      <c r="W35" s="12" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="13" t="s">
+    <row r="36" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="12" t="s">
         <v>22</v>
       </c>
       <c r="B36" s="4">
@@ -3192,81 +3337,87 @@
       <c r="T36" s="4">
         <v>5660</v>
       </c>
-      <c r="U36" s="4"/>
-      <c r="V36" s="13" t="s">
+      <c r="U36" s="4">
+        <v>5660</v>
+      </c>
+      <c r="V36" s="4"/>
+      <c r="W36" s="12" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:22" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="14" t="s">
+    <row r="37" spans="1:23" ht="17.649999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B37" s="7">
-        <v>4413</v>
-      </c>
-      <c r="C37" s="7">
+      <c r="B37" s="6">
         <v>4424</v>
       </c>
-      <c r="D37" s="7">
+      <c r="C37" s="6">
         <v>4443</v>
       </c>
-      <c r="E37" s="7">
+      <c r="D37" s="6">
         <v>4455</v>
       </c>
-      <c r="F37" s="7">
+      <c r="E37" s="6">
         <v>4478</v>
       </c>
-      <c r="G37" s="7">
+      <c r="F37" s="6">
         <v>4478</v>
       </c>
-      <c r="H37" s="7">
+      <c r="G37" s="6">
         <v>4474</v>
       </c>
-      <c r="I37" s="7">
+      <c r="H37" s="6">
         <v>4469</v>
       </c>
-      <c r="J37" s="7">
+      <c r="I37" s="6">
         <v>4462</v>
       </c>
-      <c r="K37" s="7">
+      <c r="J37" s="6">
         <v>4451</v>
       </c>
-      <c r="L37" s="7">
+      <c r="K37" s="6">
         <v>4449</v>
       </c>
-      <c r="M37" s="7">
+      <c r="L37" s="6">
         <v>4447</v>
       </c>
-      <c r="N37" s="7">
+      <c r="M37" s="6">
         <v>4439</v>
       </c>
-      <c r="O37" s="7">
+      <c r="N37" s="6">
         <v>4408</v>
       </c>
-      <c r="P37" s="7">
+      <c r="O37" s="6">
         <v>4406</v>
       </c>
-      <c r="Q37" s="7">
+      <c r="P37" s="6">
         <v>4411</v>
       </c>
-      <c r="R37" s="7">
+      <c r="Q37" s="6">
         <v>4438</v>
       </c>
-      <c r="S37" s="7">
+      <c r="R37" s="6">
         <v>4461</v>
       </c>
-      <c r="T37" s="7">
+      <c r="S37" s="6">
         <v>4563</v>
       </c>
-      <c r="U37" s="7"/>
-      <c r="V37" s="14" t="s">
+      <c r="T37" s="6">
+        <v>4656</v>
+      </c>
+      <c r="U37" s="6">
+        <v>4714</v>
+      </c>
+      <c r="V37" s="6"/>
+      <c r="W37" s="13" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="V38" s="6"/>
-    </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="W38" s="5"/>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>9</v>
       </c>
@@ -3282,8 +3433,9 @@
       <c r="S39" s="2"/>
       <c r="T39" s="2"/>
       <c r="U39" s="2"/>
-    </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="V39" s="2"/>
+    </row>
+    <row r="40" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>28</v>
       </c>
@@ -3293,14 +3445,15 @@
       <c r="M40" s="2"/>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
-      <c r="P40" s="8"/>
+      <c r="P40" s="7"/>
       <c r="Q40" s="2"/>
       <c r="R40" s="2"/>
-      <c r="S40" s="17"/>
-      <c r="T40" s="17"/>
-      <c r="U40" s="17"/>
-    </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="S40" s="16"/>
+      <c r="T40" s="16"/>
+      <c r="U40" s="16"/>
+      <c r="V40" s="16"/>
+    </row>
+    <row r="41" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>26</v>
       </c>
@@ -3310,40 +3463,42 @@
       <c r="M41" s="2"/>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
-      <c r="P41" s="8"/>
+      <c r="P41" s="7"/>
       <c r="Q41" s="2"/>
       <c r="R41" s="2"/>
       <c r="S41" s="2"/>
       <c r="T41" s="2"/>
       <c r="U41" s="2"/>
-      <c r="V41" s="6"/>
-    </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="P42" s="9"/>
-      <c r="S42" s="9"/>
-      <c r="T42" s="9"/>
-      <c r="U42" s="9"/>
-    </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="P43" s="9"/>
-    </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="P44" s="9"/>
+      <c r="V41" s="2"/>
+      <c r="W41" s="5"/>
+    </row>
+    <row r="42" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="P42" s="8"/>
+      <c r="S42" s="8"/>
+      <c r="T42" s="8"/>
+      <c r="U42" s="8"/>
+      <c r="V42" s="8"/>
+    </row>
+    <row r="43" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="P43" s="8"/>
+    </row>
+    <row r="44" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="P44" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B1:U1"/>
-    <mergeCell ref="B2:U2"/>
+    <mergeCell ref="B1:V1"/>
+    <mergeCell ref="B2:V2"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data entry" error="You can only enter  numbers" promptTitle="Data entry" prompt="Please enter a number" sqref="S40:U40" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Data entry" error="You can only enter  numbers" promptTitle="Data entry" prompt="Please enter a number" sqref="S40:V40" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>0</formula1>
       <formula2>1E+42</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.62992125984251968" bottom="0.19685039370078741" header="0.15748031496062992" footer="0.15748031496062992"/>
-  <pageSetup paperSize="8" scale="91" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="8" scale="88" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0">
     <oddHeader>&amp;R&amp;F</oddHeader>
   </headerFooter>

</xml_diff>